<commit_message>
feat: por pagar sum metric, abonos sheet in excel, and loan history modal
</commit_message>
<xml_diff>
--- a/FinFlow Bank.xlsx
+++ b/FinFlow Bank.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Ingresos" sheetId="3" r:id="rId3"/>
     <sheet name="Deudas" sheetId="4" r:id="rId4"/>
     <sheet name="Prestamos" sheetId="5" r:id="rId5"/>
+    <sheet name="Abonos" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -411,7 +412,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -530,30 +531,53 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>exp-1791069599624</v>
+        <v>exp-1792012015847</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C6" t="str">
         <v>USR-001</v>
       </c>
       <c r="D6" t="str">
-        <v>N/A</v>
+        <v>Otros</v>
       </c>
       <c r="E6" t="str">
         <v>Gastos</v>
       </c>
       <c r="F6">
-        <v>115000</v>
+        <v>65000</v>
       </c>
       <c r="G6" t="str">
         <v>Tarjeta de Débito</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>exp-1791069599624</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="C7" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="D7" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Gastos</v>
+      </c>
+      <c r="F7">
+        <v>115000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Tarjeta de Débito</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -787,7 +811,7 @@
         <v>1469000</v>
       </c>
       <c r="F5">
-        <v>73450</v>
+        <v>293800</v>
       </c>
       <c r="G5" t="str">
         <v>2027-02-28</v>
@@ -811,7 +835,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:Q5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -850,6 +874,21 @@
       <c r="L1" t="str">
         <v>Estado</v>
       </c>
+      <c r="M1" t="str">
+        <v>Total Abonos</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Último Abono</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Fecha Último Abono</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Abono 1</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Fecha 1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -888,6 +927,21 @@
       <c r="L2" t="str">
         <v>Al día</v>
       </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>600</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="P2">
+        <v>600</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>2026-08-10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -926,6 +980,21 @@
       <c r="L3" t="str">
         <v>Al día</v>
       </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>3000</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="P3">
+        <v>3000</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>2026-07-01</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -964,6 +1033,21 @@
       <c r="L4" t="str">
         <v>Al día</v>
       </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>80000</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="P4">
+        <v>80000</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>2026-10-03</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -994,18 +1078,174 @@
         <v>470000</v>
       </c>
       <c r="J5">
+        <v>1250000</v>
+      </c>
+      <c r="K5">
         <v>1100000</v>
-      </c>
-      <c r="K5">
-        <v>1250000</v>
       </c>
       <c r="L5" t="str">
         <v>Al día</v>
       </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1250000</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="P5">
+        <v>1250000</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>2026-10-03</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID Abono</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Fecha</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ID Préstamo</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Prestatario</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Monto Abonado</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Saldo Restante</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Notas</v>
+      </c>
+      <c r="H1" t="str">
+        <v>ID Usuario</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>lpay-loan-1-init</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="C2" t="str">
+        <v>loan-1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Alejandro Rivera</v>
+      </c>
+      <c r="E2">
+        <v>600</v>
+      </c>
+      <c r="F2">
+        <v>900</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Abono inicial registrado</v>
+      </c>
+      <c r="H2" t="str">
+        <v>user-carlos-2026</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>lpay-loan-2-init</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>loan-2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Fondo Emprendimiento Familiar</v>
+      </c>
+      <c r="E3">
+        <v>3000</v>
+      </c>
+      <c r="F3">
+        <v>2000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Abono inicial registrado</v>
+      </c>
+      <c r="H3" t="str">
+        <v>user-carlos-2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>lpay-1791065834687-1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="C4" t="str">
+        <v>loan-1791065834687</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Grafica - Yeison</v>
+      </c>
+      <c r="E4">
+        <v>80000</v>
+      </c>
+      <c r="F4">
+        <v>920000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Abono inicial</v>
+      </c>
+      <c r="H4" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>lpay-1791065791483-1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="C5" t="str">
+        <v>loan-1791065791483</v>
+      </c>
+      <c r="D5" t="str">
+        <v>PC Gamer - Anderson</v>
+      </c>
+      <c r="E5">
+        <v>1250000</v>
+      </c>
+      <c r="F5">
+        <v>1100000</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Abono inicial</v>
+      </c>
+      <c r="H5" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: debt abonos persistence in excel and DebtHistoryModal popup
</commit_message>
<xml_diff>
--- a/FinFlow Bank.xlsx
+++ b/FinFlow Bank.xlsx
@@ -664,7 +664,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:O5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -697,6 +697,21 @@
       <c r="J1" t="str">
         <v>Estado</v>
       </c>
+      <c r="K1" t="str">
+        <v>Total Abonos</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Último Abono</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Fecha Último Abono</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Abono 1</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Fecha 1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -729,6 +744,21 @@
       <c r="J2" t="str">
         <v>Activa</v>
       </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>7500</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="N2">
+        <v>7500</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-09-21</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -761,6 +791,21 @@
       <c r="J3" t="str">
         <v>Activa</v>
       </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>2820</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="N3">
+        <v>2820</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-09-21</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -793,6 +838,21 @@
       <c r="J4" t="str">
         <v>Activa</v>
       </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>100000</v>
+      </c>
+      <c r="M4" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="N4">
+        <v>100000</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-10-03</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -825,10 +885,25 @@
       <c r="J5" t="str">
         <v>Activa</v>
       </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>900000</v>
+      </c>
+      <c r="M5" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="N5">
+        <v>900000</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-10-03</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1111,7 +1186,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1121,21 +1196,24 @@
         <v>Fecha</v>
       </c>
       <c r="C1" t="str">
-        <v>ID Préstamo</v>
+        <v>Tipo</v>
       </c>
       <c r="D1" t="str">
-        <v>Prestatario</v>
+        <v>ID Referencia</v>
       </c>
       <c r="E1" t="str">
+        <v>Acreedor / Prestatario</v>
+      </c>
+      <c r="F1" t="str">
         <v>Monto Abonado</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Saldo Restante</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Notas</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>ID Usuario</v>
       </c>
     </row>
@@ -1147,21 +1225,24 @@
         <v>2026-08-10</v>
       </c>
       <c r="C2" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D2" t="str">
         <v>loan-1</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Alejandro Rivera</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>600</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>900</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Abono inicial registrado</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>user-carlos-2026</v>
       </c>
     </row>
@@ -1173,21 +1254,24 @@
         <v>2026-07-01</v>
       </c>
       <c r="C3" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D3" t="str">
         <v>loan-2</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Fondo Emprendimiento Familiar</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>3000</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>2000</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Abono inicial registrado</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>user-carlos-2026</v>
       </c>
     </row>
@@ -1199,21 +1283,24 @@
         <v>2026-10-03</v>
       </c>
       <c r="C4" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D4" t="str">
         <v>loan-1791065834687</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Grafica - Yeison</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>80000</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>920000</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Abono inicial</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>USR-001</v>
       </c>
     </row>
@@ -1225,27 +1312,146 @@
         <v>2026-10-03</v>
       </c>
       <c r="C5" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D5" t="str">
         <v>loan-1791065791483</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>PC Gamer - Anderson</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>1250000</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>1100000</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Abono inicial</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>dpay-debt-1-init</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D6" t="str">
+        <v>debt-1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Banco Nacional Tech</v>
+      </c>
+      <c r="F6">
+        <v>7500</v>
+      </c>
+      <c r="G6">
+        <v>14500</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Abono amortizado registrado</v>
+      </c>
+      <c r="I6" t="str">
+        <v>user-carlos-2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>dpay-debt-2-init</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D7" t="str">
+        <v>debt-2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>NeoBank Global</v>
+      </c>
+      <c r="F7">
+        <v>2820</v>
+      </c>
+      <c r="G7">
+        <v>980</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Abono amortizado registrado</v>
+      </c>
+      <c r="I7" t="str">
+        <v>user-carlos-2026</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>dpay-1791069501081-1</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D8" t="str">
+        <v>debt-1791069501081</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Lapida Mamita</v>
+      </c>
+      <c r="F8">
+        <v>100000</v>
+      </c>
+      <c r="G8">
+        <v>1500000</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Abono inicial amortizado</v>
+      </c>
+      <c r="I8" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>dpay-1791065999572-1</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D9" t="str">
+        <v>debt-1791065999572</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Institución/Persona</v>
+      </c>
+      <c r="F9">
+        <v>900000</v>
+      </c>
+      <c r="G9">
+        <v>569000</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Abono inicial amortizado</v>
+      </c>
+      <c r="I9" t="str">
         <v>USR-001</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: proteger registros historicos inmutables
</commit_message>
<xml_diff>
--- a/FinFlow Bank.xlsx
+++ b/FinFlow Bank.xlsx
@@ -1100,28 +1100,28 @@
         <v>200000</v>
       </c>
       <c r="J4">
-        <v>80000</v>
+        <v>1000000</v>
       </c>
       <c r="K4">
-        <v>920000</v>
+        <v>0</v>
       </c>
       <c r="L4" t="str">
-        <v>Al día</v>
+        <v>Saldado</v>
       </c>
       <c r="M4">
         <v>1</v>
       </c>
       <c r="N4">
-        <v>80000</v>
+        <v>920000</v>
       </c>
       <c r="O4" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
       <c r="P4">
-        <v>80000</v>
+        <v>920000</v>
       </c>
       <c r="Q4" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
     </row>
     <row r="5">
@@ -1153,10 +1153,10 @@
         <v>470000</v>
       </c>
       <c r="J5">
+        <v>1100000</v>
+      </c>
+      <c r="K5">
         <v>1250000</v>
-      </c>
-      <c r="K5">
-        <v>1100000</v>
       </c>
       <c r="L5" t="str">
         <v>Al día</v>
@@ -1186,7 +1186,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1449,9 +1449,38 @@
         <v>USR-001</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>lpay-1792014650669</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D10" t="str">
+        <v>loan-1791065834687</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Grafica - Yeison</v>
+      </c>
+      <c r="F10">
+        <v>920000</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Cobro Totalmente Recuperado</v>
+      </c>
+      <c r="I10" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: registrar nuevos usuarios en hoja Usuarios de excel sin tipo de moneda y limpiar formulario al reabrir
</commit_message>
<xml_diff>
--- a/FinFlow Bank.xlsx
+++ b/FinFlow Bank.xlsx
@@ -402,10 +402,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:H6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID Usuario</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Usuario</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Nombre Completo</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Correo</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Contraseña</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Rol</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Estado</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Fecha de Registro</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Jorge00</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Jorge Luis Perez Acosta</v>
+      </c>
+      <c r="D2" t="str">
+        <v>jorge00@finflow.io</v>
+      </c>
+      <c r="E2" t="str">
+        <v>9876**</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2026-09-20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>USR-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Sara01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Sara Morales Buitrago</v>
+      </c>
+      <c r="D3" t="str">
+        <v>sara01@finflow.io</v>
+      </c>
+      <c r="E3" t="str">
+        <v>12345</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Cliente</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-09-20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Karen02</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Karen Lorena Perez Acosta</v>
+      </c>
+      <c r="D4" t="str">
+        <v>karen02@finflow.io</v>
+      </c>
+      <c r="E4" t="str">
+        <v>12345</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Cliente</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-09-20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>USR-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Jose03</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Joselin Alverto Perez Ochoa</v>
+      </c>
+      <c r="D5" t="str">
+        <v>jose03@finflow.io</v>
+      </c>
+      <c r="E5" t="str">
+        <v>12345</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Cliente</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-09-20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>user-1792019891643</v>
+      </c>
+      <c r="B6" t="str">
+        <v>prueba</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Camilo</v>
+      </c>
+      <c r="D6" t="str">
+        <v>prueba@finflow.io</v>
+      </c>
+      <c r="E6" t="str">
+        <v>09876</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Cliente</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-10-14</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -531,7 +688,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>exp-1792012015847</v>
+        <v>exp-1792018682249</v>
       </c>
       <c r="B6" t="str">
         <v>2026-10-14</v>
@@ -554,22 +711,22 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>exp-1791069599624</v>
+        <v>exp-1792018633212</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C7" t="str">
         <v>USR-001</v>
       </c>
       <c r="D7" t="str">
-        <v>N/A</v>
+        <v>Otros</v>
       </c>
       <c r="E7" t="str">
         <v>Gastos</v>
       </c>
       <c r="F7">
-        <v>115000</v>
+        <v>115000.00000000001</v>
       </c>
       <c r="G7" t="str">
         <v>Tarjeta de Débito</v>
@@ -664,7 +821,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:Q5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -712,6 +869,12 @@
       <c r="O1" t="str">
         <v>Fecha 1</v>
       </c>
+      <c r="P1" t="str">
+        <v>Abono 2</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Fecha 2</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -809,72 +972,78 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>debt-1791069501081</v>
+        <v>debt-1792018406201</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-03</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C4" t="str">
         <v>USR-001</v>
       </c>
       <c r="D4" t="str">
-        <v>Lapida Mamita</v>
+        <v xml:space="preserve">Lapida Mamita </v>
       </c>
       <c r="E4">
         <v>1600000</v>
       </c>
       <c r="F4">
-        <v>533333</v>
+        <v>266667</v>
       </c>
       <c r="G4" t="str">
         <v>2026-12-31</v>
       </c>
       <c r="H4">
-        <v>100000</v>
+        <v>1060000</v>
       </c>
       <c r="I4">
-        <v>1500000</v>
+        <v>540000.0000000001</v>
       </c>
       <c r="J4" t="str">
         <v>Activa</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L4">
         <v>100000</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
       <c r="N4">
+        <v>959999.9999999999</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="P4">
         <v>100000</v>
       </c>
-      <c r="O4" t="str">
-        <v>2026-10-03</v>
+      <c r="Q4" t="str">
+        <v>2026-10-14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>debt-1791065999572</v>
+        <v>debt-1792018339574</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-03</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C5" t="str">
         <v>USR-001</v>
       </c>
       <c r="D5" t="str">
-        <v>Institución/Persona</v>
+        <v>Deuda Taren</v>
       </c>
       <c r="E5">
         <v>1469000</v>
       </c>
       <c r="F5">
-        <v>293800</v>
+        <v>244833</v>
       </c>
       <c r="G5" t="str">
-        <v>2027-02-28</v>
+        <v>2026-12-31</v>
       </c>
       <c r="H5">
         <v>900000</v>
@@ -892,289 +1061,13 @@
         <v>900000</v>
       </c>
       <c r="M5" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
       <c r="N5">
         <v>900000</v>
       </c>
       <c r="O5" t="str">
-        <v>2026-10-03</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O5"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q5"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID Préstamo</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Fecha Inicio</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Fecha Final</v>
-      </c>
-      <c r="D1" t="str">
-        <v>ID Usuario</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Prestatario</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Monto Prestado</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Tasa de Interés</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Plazo en Meses</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Cuota Mensual</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Monto Cobrado</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Saldo Pendiente</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Estado</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Total Abonos</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Último Abono</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Fecha Último Abono</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Abono 1</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Fecha 1</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>loan-1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2026-08-10</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2026-10-15</v>
-      </c>
-      <c r="D2" t="str">
-        <v>user-carlos-2026</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Alejandro Rivera</v>
-      </c>
-      <c r="F2">
-        <v>1500</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>750</v>
-      </c>
-      <c r="J2">
-        <v>600</v>
-      </c>
-      <c r="K2">
-        <v>900</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Al día</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>600</v>
-      </c>
-      <c r="O2" t="str">
-        <v>2026-08-10</v>
-      </c>
-      <c r="P2">
-        <v>600</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>2026-08-10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>loan-2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="C3" t="str">
-        <v>2026-11-30</v>
-      </c>
-      <c r="D3" t="str">
-        <v>user-carlos-2026</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Fondo Emprendimiento Familiar</v>
-      </c>
-      <c r="F3">
-        <v>5000</v>
-      </c>
-      <c r="G3">
-        <v>3.5</v>
-      </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
-      <c r="I3">
-        <v>1000</v>
-      </c>
-      <c r="J3">
-        <v>3000</v>
-      </c>
-      <c r="K3">
-        <v>2000</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Al día</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>3000</v>
-      </c>
-      <c r="O3" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="P3">
-        <v>3000</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>2026-07-01</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>loan-1791065834687</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-10-03</v>
-      </c>
-      <c r="C4" t="str">
-        <v>2027-02-28</v>
-      </c>
-      <c r="D4" t="str">
-        <v>USR-001</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Grafica - Yeison</v>
-      </c>
-      <c r="F4">
-        <v>1000000</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>5</v>
-      </c>
-      <c r="I4">
-        <v>200000</v>
-      </c>
-      <c r="J4">
-        <v>1000000</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Saldado</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-      <c r="N4">
-        <v>920000</v>
-      </c>
-      <c r="O4" t="str">
-        <v>2026-10-14</v>
-      </c>
-      <c r="P4">
-        <v>920000</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>2026-10-14</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>loan-1791065791483</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-10-03</v>
-      </c>
-      <c r="C5" t="str">
-        <v>2027-02-28</v>
-      </c>
-      <c r="D5" t="str">
-        <v>USR-001</v>
-      </c>
-      <c r="E5" t="str">
-        <v>PC Gamer - Anderson</v>
-      </c>
-      <c r="F5">
-        <v>2350000</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>5</v>
-      </c>
-      <c r="I5">
-        <v>470000</v>
-      </c>
-      <c r="J5">
-        <v>1100000</v>
-      </c>
-      <c r="K5">
-        <v>1250000</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Al día</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5">
-        <v>1250000</v>
-      </c>
-      <c r="O5" t="str">
-        <v>2026-10-03</v>
-      </c>
-      <c r="P5">
-        <v>1250000</v>
-      </c>
-      <c r="Q5" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-14</v>
       </c>
     </row>
   </sheetData>
@@ -1184,9 +1077,303 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:S5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID Préstamo</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Fecha Inicio</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Fecha Final</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ID Usuario</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Prestatario</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Monto Prestado</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tasa de Interés</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Plazo en Meses</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Cuota Mensual</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Monto Cobrado</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Saldo Pendiente</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Estado</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Total Abonos</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Último Abono</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Fecha Último Abono</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Abono 1</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Fecha 1</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Abono 2</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Fecha 2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>loan-1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-10-15</v>
+      </c>
+      <c r="D2" t="str">
+        <v>user-carlos-2026</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Alejandro Rivera</v>
+      </c>
+      <c r="F2">
+        <v>1500</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>750</v>
+      </c>
+      <c r="J2">
+        <v>600</v>
+      </c>
+      <c r="K2">
+        <v>900</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Al día</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>600</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="P2">
+        <v>600</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>2026-08-10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>loan-2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-11-30</v>
+      </c>
+      <c r="D3" t="str">
+        <v>user-carlos-2026</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Fondo Emprendimiento Familiar</v>
+      </c>
+      <c r="F3">
+        <v>5000</v>
+      </c>
+      <c r="G3">
+        <v>3.5</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>1000</v>
+      </c>
+      <c r="J3">
+        <v>3000</v>
+      </c>
+      <c r="K3">
+        <v>2000</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Al día</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>3000</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="P3">
+        <v>3000</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>loan-1792018163585</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="D4" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E4" t="str">
+        <v>PC Gamer Anderson</v>
+      </c>
+      <c r="F4">
+        <v>2350000</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="I4">
+        <v>391667</v>
+      </c>
+      <c r="J4">
+        <v>1100000</v>
+      </c>
+      <c r="K4">
+        <v>1250000</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Al día</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4">
+        <v>100000</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="P4">
+        <v>1000000</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="R4">
+        <v>100000</v>
+      </c>
+      <c r="S4" t="str">
+        <v>2026-10-14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>loan-1792018095098</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="D5" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Grafica Yeison</v>
+      </c>
+      <c r="F5">
+        <v>1000000</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>200000</v>
+      </c>
+      <c r="J5">
+        <v>80000</v>
+      </c>
+      <c r="K5">
+        <v>920000</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Al día</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+      <c r="N5">
+        <v>14999.999999999998</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="P5">
+        <v>65000</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="R5">
+        <v>14999.999999999998</v>
+      </c>
+      <c r="S5" t="str">
+        <v>2026-10-14</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:S5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1478,9 +1665,212 @@
         <v>USR-001</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>lpay-1792018193842</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D11" t="str">
+        <v>loan-1792018095098</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Grafica Yeison</v>
+      </c>
+      <c r="F11">
+        <v>65000</v>
+      </c>
+      <c r="G11">
+        <v>920000</v>
+      </c>
+      <c r="H11" t="str">
+        <v xml:space="preserve">Transferencia </v>
+      </c>
+      <c r="I11" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>lpay-1792018209544</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D12" t="str">
+        <v>loan-1792018095098</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Grafica Yeison</v>
+      </c>
+      <c r="F12">
+        <v>14999.999999999998</v>
+      </c>
+      <c r="G12">
+        <v>920000</v>
+      </c>
+      <c r="H12" t="str">
+        <v xml:space="preserve">Efectivo </v>
+      </c>
+      <c r="I12" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>lpay-1792018237315</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D13" t="str">
+        <v>loan-1792018163585</v>
+      </c>
+      <c r="E13" t="str">
+        <v>PC Gamer Anderson</v>
+      </c>
+      <c r="F13">
+        <v>1000000</v>
+      </c>
+      <c r="G13">
+        <v>1250000</v>
+      </c>
+      <c r="H13" t="str">
+        <v xml:space="preserve">Efectivo </v>
+      </c>
+      <c r="I13" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>lpay-1792018248654</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Préstamo</v>
+      </c>
+      <c r="D14" t="str">
+        <v>loan-1792018163585</v>
+      </c>
+      <c r="E14" t="str">
+        <v>PC Gamer Anderson</v>
+      </c>
+      <c r="F14">
+        <v>100000</v>
+      </c>
+      <c r="G14">
+        <v>1250000</v>
+      </c>
+      <c r="H14" t="str">
+        <v xml:space="preserve">Efectivo </v>
+      </c>
+      <c r="I14" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>pay-1792018492817</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D15" t="str">
+        <v>debt-1792018406201</v>
+      </c>
+      <c r="E15" t="str">
+        <v xml:space="preserve">Lapida Mamita </v>
+      </c>
+      <c r="F15">
+        <v>959999.9999999999</v>
+      </c>
+      <c r="G15">
+        <v>540000.0000000001</v>
+      </c>
+      <c r="H15" t="str">
+        <v xml:space="preserve">Efectivo </v>
+      </c>
+      <c r="I15" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>pay-1792018513671</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D16" t="str">
+        <v>debt-1792018406201</v>
+      </c>
+      <c r="E16" t="str">
+        <v xml:space="preserve">Lapida Mamita </v>
+      </c>
+      <c r="F16">
+        <v>100000</v>
+      </c>
+      <c r="G16">
+        <v>540000.0000000001</v>
+      </c>
+      <c r="H16" t="str">
+        <v xml:space="preserve">Efectivo </v>
+      </c>
+      <c r="I16" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>pay-1792018580790</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D17" t="str">
+        <v>debt-1792018339574</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Deuda Taren</v>
+      </c>
+      <c r="F17">
+        <v>900000</v>
+      </c>
+      <c r="G17">
+        <v>569000</v>
+      </c>
+      <c r="H17" t="str">
+        <v xml:space="preserve">Efectivo </v>
+      </c>
+      <c r="I17" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: registrar nuevos usuarios en hoja Usuarios de Google Sheets y auto-sincronizar
</commit_message>
<xml_diff>
--- a/FinFlow Bank.xlsx
+++ b/FinFlow Bank.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -560,9 +560,35 @@
         <v>2026-10-14</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>user-1792021015402</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Prueba</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Camilo</v>
+      </c>
+      <c r="D7" t="str">
+        <v>prueba@gmail.com</v>
+      </c>
+      <c r="E7" t="str">
+        <v>123456123456</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Cliente</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-10-14</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: diferenciacio visual permanente de abonos y aumentos de deuda/prestamo con registro individual
</commit_message>
<xml_diff>
--- a/FinFlow Bank.xlsx
+++ b/FinFlow Bank.xlsx
@@ -847,7 +847,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:S6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -901,6 +901,12 @@
       <c r="Q1" t="str">
         <v>Fecha 2</v>
       </c>
+      <c r="R1" t="str">
+        <v>Abono 3</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Fecha 3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -998,60 +1004,48 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>debt-1792018406201</v>
+        <v>debt-1792376292618</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-07-01</v>
+        <v>2026-10-19</v>
       </c>
       <c r="C4" t="str">
         <v>USR-001</v>
       </c>
       <c r="D4" t="str">
-        <v xml:space="preserve">Lapida Mamita </v>
+        <v xml:space="preserve">Inyección Anticonceptiva </v>
       </c>
       <c r="E4">
-        <v>1600000</v>
+        <v>30000</v>
       </c>
       <c r="F4">
-        <v>266667</v>
+        <v>30000</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-12-31</v>
+        <v>2026-10-23</v>
       </c>
       <c r="H4">
-        <v>1060000</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>540000.0000000001</v>
+        <v>30000</v>
       </c>
       <c r="J4" t="str">
         <v>Activa</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-10-14</v>
-      </c>
-      <c r="N4">
-        <v>959999.9999999999</v>
-      </c>
-      <c r="O4" t="str">
-        <v>2026-10-14</v>
-      </c>
-      <c r="P4">
-        <v>100000</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>2026-10-14</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>debt-1792018339574</v>
+        <v>debt-1792018406201</v>
       </c>
       <c r="B5" t="str">
         <v>2026-07-01</v>
@@ -1060,22 +1054,22 @@
         <v>USR-001</v>
       </c>
       <c r="D5" t="str">
-        <v>Deuda Taren</v>
+        <v xml:space="preserve">Lapida Mamita </v>
       </c>
       <c r="E5">
-        <v>1469000</v>
+        <v>1600000</v>
       </c>
       <c r="F5">
-        <v>244833</v>
+        <v>266667</v>
       </c>
       <c r="G5" t="str">
         <v>2026-12-31</v>
       </c>
       <c r="H5">
-        <v>900000</v>
+        <v>1110000</v>
       </c>
       <c r="I5">
-        <v>569000</v>
+        <v>490000.0000000001</v>
       </c>
       <c r="J5" t="str">
         <v>Activa</v>
@@ -1084,21 +1078,80 @@
         <v>1</v>
       </c>
       <c r="L5">
+        <v>1110000</v>
+      </c>
+      <c r="M5" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="N5">
+        <v>1110000</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>debt-1792018339574</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Deuda Taren</v>
+      </c>
+      <c r="E6">
+        <v>1524000</v>
+      </c>
+      <c r="F6">
+        <v>254000</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="H6">
         <v>900000</v>
       </c>
-      <c r="M5" t="str">
-        <v>2026-10-14</v>
-      </c>
-      <c r="N5">
+      <c r="I6">
+        <v>624000</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Activa</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>22000</v>
+      </c>
+      <c r="M6" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="N6">
         <v>900000</v>
       </c>
-      <c r="O5" t="str">
-        <v>2026-10-14</v>
+      <c r="O6" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="P6">
+        <v>33000</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="R6">
+        <v>22000</v>
+      </c>
+      <c r="S6" t="str">
+        <v>2026-10-19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1399,7 +1452,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1894,9 +1947,125 @@
         <v>USR-001</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>dpay-debt-1792018406201-init</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D18" t="str">
+        <v>debt-1792018406201</v>
+      </c>
+      <c r="E18" t="str">
+        <v xml:space="preserve">Lapida Mamita </v>
+      </c>
+      <c r="F18">
+        <v>1110000</v>
+      </c>
+      <c r="G18">
+        <v>490000.0000000001</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Abono inicial registrado</v>
+      </c>
+      <c r="I18" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>dpay-debt-1792018339574-init</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D19" t="str">
+        <v>debt-1792018339574</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Deuda Taren</v>
+      </c>
+      <c r="F19">
+        <v>900000</v>
+      </c>
+      <c r="G19">
+        <v>624000</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Abono inicial registrado</v>
+      </c>
+      <c r="I19" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>inc-1792380521660</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D20" t="str">
+        <v>debt-1792018339574</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Deuda Taren</v>
+      </c>
+      <c r="F20">
+        <v>33000</v>
+      </c>
+      <c r="G20">
+        <v>624000</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Cumpleaños Mamá Nena</v>
+      </c>
+      <c r="I20" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>inc-1792380559489</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Deuda</v>
+      </c>
+      <c r="D21" t="str">
+        <v>debt-1792018339574</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Deuda Taren</v>
+      </c>
+      <c r="F21">
+        <v>22000</v>
+      </c>
+      <c r="G21">
+        <v>624000</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Pesas Moto</v>
+      </c>
+      <c r="I21" t="str">
+        <v>USR-001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>